<commit_message>
subida de json echo con excel-01
genere un quiz desde excel con python y  los assests creados son el archivo json bio test 01 y la actualización del index.
</commit_message>
<xml_diff>
--- a/excel/test-excel-1.xlsx
+++ b/excel/test-excel-1.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e6cea8a9fac91e1a/Documentos/Excel-json-github-bg/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\dev\biogenios-db\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="11_F25DC773A252ABDACC10488B199970DA5BDE58E9" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{62D0CC2A-29AD-49C5-9385-CCFE90504431}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DACB87A-EDDB-4506-867F-AD7A1A909491}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,27 +37,15 @@
     <t>id_index</t>
   </si>
   <si>
-    <t>bio_general_01</t>
-  </si>
-  <si>
     <t>titulo</t>
   </si>
   <si>
-    <t>Biología General – UNSCH (Ciclo Verano)</t>
-  </si>
-  <si>
     <t>tema</t>
   </si>
   <si>
-    <t>Biología Rumbo a la UNSCH - Ciclo Verano</t>
-  </si>
-  <si>
     <t>descripcion</t>
   </si>
   <si>
-    <t>Simulacro tipo admisión con preguntas frecuentes</t>
-  </si>
-  <si>
     <t>area</t>
   </si>
   <si>
@@ -67,15 +55,9 @@
     <t>nivel</t>
   </si>
   <si>
-    <t>Admisión</t>
-  </si>
-  <si>
     <t>archivo</t>
   </si>
   <si>
-    <t>biologia/biologia_general_01.json</t>
-  </si>
-  <si>
     <t>id</t>
   </si>
   <si>
@@ -134,6 +116,24 @@
   </si>
   <si>
     <t>Vacuola</t>
+  </si>
+  <si>
+    <t>bio_test_01</t>
+  </si>
+  <si>
+    <t>fast test para pruebas del programa</t>
+  </si>
+  <si>
+    <t>Pre Biología semana 04</t>
+  </si>
+  <si>
+    <t>Simulacro tipo admisión con preguntas frecuentes ciclo verano semana 04</t>
+  </si>
+  <si>
+    <t>ETA-test-01</t>
+  </si>
+  <si>
+    <t>biologia/bio_test_01.json</t>
   </si>
 </sst>
 </file>
@@ -485,55 +485,55 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>3</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>5</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>7</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -548,28 +548,28 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
@@ -577,25 +577,25 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -603,25 +603,25 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>